<commit_message>
Build publications site; include self-author name at correct position in bylines
</commit_message>
<xml_diff>
--- a/data/publications.xlsx
+++ b/data/publications.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Co-authors</t>
+          <t>Authors</t>
         </is>
       </c>
     </row>
@@ -480,7 +480,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Miranda C. Mudge; Michael Riffle; Gabriella Chebli; Deanna L. Plubell; Tatiana A. Rynearson; William Stafford Noble; Julia Kubanek; Brook L. Nunn</t>
+          <t>Miranda C. Mudge; Michael Riffle; Gabriella Chebli; Deanna L. Plubell; Tatiana A. Rynearson; William Stafford Noble; Emma Timmins‐Schiffman; Julia Kubanek; Brook L. Nunn</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Josep V. Planas; Andrew Jasonowicz; Anna Simeon; Crystal Simchick; Brook L. Nunn; Anita C. Kroska; Nathan Wolf; Thomas P. Hurst</t>
+          <t>Josep V. Planas; Andrew Jasonowicz; Anna Simeon; Crystal Simchick; Emma Timmins‐Schiffman; Brook L. Nunn; Anita C. Kroska; Nathan Wolf; Thomas P. Hurst</t>
         </is>
       </c>
     </row>
@@ -530,7 +530,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Larken Root; Ryan Crim; Mollie A. Middleton; Megan M. Ewing; Jacob R. Winnikoff; Gracelyn Ham; Giles Goetz; Steven Roberts; Mackenzie Gavery</t>
+          <t>Emma Timmins‐Schiffman; Larken Root; Ryan Crim; Mollie A. Middleton; Megan M. Ewing; Jacob R. Winnikoff; Gracelyn Ham; Giles Goetz; Steven Roberts; Mackenzie Gavery</t>
         </is>
       </c>
     </row>
@@ -555,7 +555,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Brook L. Nunn; Tanya Brown; Miranda C. Mudge; Michael Riffle; Jeremy B. Axworthy; Jenna Dilworth; Carly D. Kenkel; Jesse Zaneveld; Lisa J. Rodrigues; Jacqueline L. Padilla‐Gamiño</t>
+          <t>Brook L. Nunn; Tanya Brown; Emma Timmins‐Schiffman; Miranda C. Mudge; Michael Riffle; Jeremy B. Axworthy; Jenna Dilworth; Carly D. Kenkel; Jesse Zaneveld; Lisa J. Rodrigues; Jacqueline L. Padilla‐Gamiño</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Anais S. Gentilhomme; Kusum Dhakar; Matthew Chaw; Erin Firth; Karen Junge; Brook L. Nunn</t>
+          <t>Anais S. Gentilhomme; Kusum Dhakar; Emma Timmins‐Schiffman; Matthew Chaw; Erin Firth; Karen Junge; Brook L. Nunn</t>
         </is>
       </c>
     </row>
@@ -605,7 +605,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Rayhan Khanna; Tanya Brown; Jenna Dilworth; Brendan MacLean; Miranda C. Mudge; Samuel J. White; Carly D. Kenkel; Lisa J. Rodrigues; Brook L. Nunn; Jacqueline L. Padilla‐Gamiño</t>
+          <t>Emma Timmins‐Schiffman; Rayhan Khanna; Tanya Brown; Jenna Dilworth; Brendan MacLean; Miranda C. Mudge; Samuel J. White; Carly D. Kenkel; Lisa J. Rodrigues; Brook L. Nunn; Jacqueline L. Padilla‐Gamiño</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Jennifer Telish; Chelsea Field; Chris Monson; José M. Guzmán; Brook L. Nunn; Graham Young; Kristy L. Forsgren</t>
+          <t>Emma Timmins‐Schiffman; Jennifer Telish; Chelsea Field; Chris Monson; José M. Guzmán; Brook L. Nunn; Graham Young; Kristy L. Forsgren</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Amy M. Van Cise; Alexandra D. Switzer; Amy Apprill; Cory D. Champagne; Paul M. Chittaro; Natasha K. Dudek; Mackenzie Gavery; Brittany L. Hancock‐Hanser; Alaina Harmon; Alexander L. Jaffe; Nicholas M. Kellar; Carolyn A. Miller; Phillip A. Morin; Sarah E. Nelms; Kelly M. Robertson; Irvin R. Schultz; Ebru Ünal; Kim M. Parsons</t>
+          <t>Amy M. Van Cise; Alexandra D. Switzer; Amy Apprill; Cory D. Champagne; Paul M. Chittaro; Natasha K. Dudek; Mackenzie Gavery; Brittany L. Hancock‐Hanser; Alaina Harmon; Alexander L. Jaffe; Nicholas M. Kellar; Carolyn A. Miller; Phillip A. Morin; Sarah E. Nelms; Kelly M. Robertson; Irvin R. Schultz; Emma Timmins‐Schiffman; Ebru Ünal; Kim M. Parsons</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Amy E. Maas; Ann M. Tarrant; Brook L. Nunn; Jea Park; Leocadio Blanco‐Bercial</t>
+          <t>Amy E. Maas; Emma Timmins‐Schiffman; Ann M. Tarrant; Brook L. Nunn; Jea Park; Leocadio Blanco‐Bercial</t>
         </is>
       </c>
     </row>
@@ -705,7 +705,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Brook L. Nunn; Miranda C. Mudge; Deanna L. Plubell; Gabriella Chebli; Julia Kubanek; Michael Riffle; William Stafford Noble; Elizabeth L. Harvey; Tasman A. Nunn; Tatiana Rynearson; Marcel Huntemann; Kurt LaButti; Brian Foster; Bryce Foster; Simon Roux; Krishna Palaniappan; Supratim Mukherjee; T. B. K. Reddy; Chris Daum; Alex Copeland; I-Min A. Chen; Natalia Ivanova; Nikos C. Kyrpides; Tijana Glavina del Rio; Emiley A. Eloe‐Fadrosh</t>
+          <t>Brook L. Nunn; Emma Timmins‐Schiffman; Miranda C. Mudge; Deanna L. Plubell; Gabriella Chebli; Julia Kubanek; Michael Riffle; William Stafford Noble; Elizabeth L. Harvey; Tasman A. Nunn; Tatiana Rynearson; Marcel Huntemann; Kurt LaButti; Brian Foster; Bryce Foster; Simon Roux; Krishna Palaniappan; Supratim Mukherjee; T. B. K. Reddy; Chris Daum; Alex Copeland; I-Min A. Chen; Natalia Ivanova; Nikos C. Kyrpides; Tijana Glavina del Rio; Emiley A. Eloe‐Fadrosh</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Amy E. Maas; Rayhan Khanna; Leocadio Blanco‐Bercial; Eric Huang; Brook L. Nunn</t>
+          <t>Emma Timmins‐Schiffman; Amy E. Maas; Rayhan Khanna; Leocadio Blanco‐Bercial; Eric Huang; Brook L. Nunn</t>
         </is>
       </c>
     </row>
@@ -755,7 +755,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>E Duselis; Tony Brown; J B Axworthy; C H Backstrom; Michael Riffle; J.R. Dilworth; Carly D. Kenkel; Lisa J. Rodrigues; Brook L. Nunn; Jacqueline L. Padilla‐Gamiño</t>
+          <t>Emma Timmins‐Schiffman; E Duselis; Tony Brown; J B Axworthy; C H Backstrom; Michael Riffle; J.R. Dilworth; Carly D. Kenkel; Lisa J. Rodrigues; Brook L. Nunn; Jacqueline L. Padilla‐Gamiño</t>
         </is>
       </c>
     </row>
@@ -780,7 +780,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Jiro Tsuchiya; Sayaka Mino; Fuki Fujiwara; Nao Okuma; Yasunori Ichihashi; Robert M. Morris; Brook L. Nunn; Tomoo Sawabe</t>
+          <t>Jiro Tsuchiya; Sayaka Mino; Fuki Fujiwara; Nao Okuma; Yasunori Ichihashi; Robert M. Morris; Brook L. Nunn; Emma Timmins‐Schiffman; Tomoo Sawabe</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Grace Crandall; Rhonda Elliott Thompson; Benoït Eudeline; Brent Vadopalas; Steven Roberts</t>
+          <t>Grace Crandall; Rhonda Elliott Thompson; Benoït Eudeline; Brent Vadopalas; Emma Timmins‐Schiffman; Steven Roberts</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Jeremy B. Axworthy; Tanya Brown; Lisa J. Rodrigues; Brook L. Nunn; Jacqueline L. Padilla‐Gamiño</t>
+          <t>Jeremy B. Axworthy; Emma Timmins‐Schiffman; Tanya Brown; Lisa J. Rodrigues; Brook L. Nunn; Jacqueline L. Padilla‐Gamiño</t>
         </is>
       </c>
     </row>
@@ -855,7 +855,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Philip W. Boyd; Scott C. Doney; Sam Eggins; Michael J. Ellwood; Marion Fourquez; Brook L. Nunn; Robert F. Strzepek</t>
+          <t>Philip W. Boyd; Scott C. Doney; Sam Eggins; Michael J. Ellwood; Marion Fourquez; Brook L. Nunn; Robert F. Strzepek; Emma Timmins‐Schiffman</t>
         </is>
       </c>
     </row>
@@ -880,7 +880,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Samuel J. White; Rhonda Elliott Thompson; Brent Vadopalas; Benoït Eudeline; Brook L. Nunn; Steven Roberts</t>
+          <t>Emma Timmins‐Schiffman; Samuel J. White; Rhonda Elliott Thompson; Brent Vadopalas; Benoït Eudeline; Brook L. Nunn; Steven Roberts</t>
         </is>
       </c>
     </row>
@@ -905,7 +905,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Kaho H. Tisthammer; François Seneca; Brook L. Nunn; Robert H. Richmond</t>
+          <t>Kaho H. Tisthammer; Emma Timmins‐Schiffman; François Seneca; Brook L. Nunn; Robert H. Richmond</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>José M. Guzmán; Rhonda Elliott Thompson; Brent Vadopalas; Benoït Eudeline; Steven Roberts</t>
+          <t>Emma Timmins‐Schiffman; José M. Guzmán; Rhonda Elliott Thompson; Brent Vadopalas; Benoït Eudeline; Steven Roberts</t>
         </is>
       </c>
     </row>
@@ -955,7 +955,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Shelly A. Wanamaker; Kaitlyn R. Mitchell; Rhonda Elliott Thompson; Benoït Eudeline; Brent Vadopalas; Steven Roberts</t>
+          <t>Shelly A. Wanamaker; Kaitlyn R. Mitchell; Rhonda Elliott Thompson; Benoït Eudeline; Brent Vadopalas; Emma Timmins‐Schiffman; Steven Roberts</t>
         </is>
       </c>
     </row>
@@ -980,7 +980,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Yaamini R. Venkataraman; MJ Horwith; AT Lowe; Brook L. Nunn; Brent Vadopalas; LH Spencer; Steven Roberts</t>
+          <t>Yaamini R. Venkataraman; Emma Timmins‐Schiffman; MJ Horwith; AT Lowe; Brook L. Nunn; Brent Vadopalas; LH Spencer; Steven Roberts</t>
         </is>
       </c>
     </row>
@@ -1005,7 +1005,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>José M. Guzmán; Rhonda Elliott Thompson; Brent Vadopalas; Benoït Eudeline; Steven Roberts</t>
+          <t>Emma Timmins‐Schiffman; José M. Guzmán; Rhonda Elliott Thompson; Brent Vadopalas; Benoït Eudeline; Steven Roberts</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Dasha Krayushkina; Jessica Faux; Damon May; Michael Riffle; H. Rodger Harvey; Brook L. Nunn</t>
+          <t>Dasha Krayushkina; Emma Timmins‐Schiffman; Jessica Faux; Damon May; Michael Riffle; H. Rodger Harvey; Brook L. Nunn</t>
         </is>
       </c>
     </row>
@@ -1055,7 +1055,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Molly P. Mikan; H. Rodger Harvey; Michael Riffle; Damon May; Ian Salter; William Stafford Noble; Brook L. Nunn</t>
+          <t>Molly P. Mikan; H. Rodger Harvey; Emma Timmins‐Schiffman; Michael Riffle; Damon May; Ian Salter; William Stafford Noble; Brook L. Nunn</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1080,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Laura H. Spencer; Micah Horwith; Alexander T. Lowe; Yaamini R. Venkataraman; Brook L. Nunn; Steven Roberts</t>
+          <t>Laura H. Spencer; Micah Horwith; Alexander T. Lowe; Yaamini R. Venkataraman; Emma Timmins‐Schiffman; Brook L. Nunn; Steven Roberts</t>
         </is>
       </c>
     </row>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Molly P. Mikan; Ying S. Ting; H. Rodger Harvey; Brook L. Nunn</t>
+          <t>Emma Timmins‐Schiffman; Molly P. Mikan; Ying S. Ting; H. Rodger Harvey; Brook L. Nunn</t>
         </is>
       </c>
     </row>
@@ -1130,7 +1130,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Amy E. Maas; Leocadio Blanco‐Bercial; Ali Lo; Ann M. Tarrant</t>
+          <t>Amy E. Maas; Leocadio Blanco‐Bercial; Ali Lo; Ann M. Tarrant; Emma Timmins‐Schiffman</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1155,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Marie-Caroline Smith; Monika Coton; Emmanuel Coton; Nolwenn Hymery; Brook L. Nunn; Stéphanie Madec</t>
+          <t>Marie-Caroline Smith; Emma Timmins‐Schiffman; Monika Coton; Emmanuel Coton; Nolwenn Hymery; Brook L. Nunn; Stéphanie Madec</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Robin S. Waples; Anna Elz; Billy D. Arnsberg; James R. Faulkner; Jeffrey J. Hard; Linda K. Park</t>
+          <t>Robin S. Waples; Anna Elz; Billy D. Arnsberg; James R. Faulkner; Jeffrey J. Hard; Emma Timmins‐Schiffman; Linda K. Park</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1205,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Grace Crandall; Brent Vadopalas; Michael Riffle; Brook L. Nunn; Steven Roberts</t>
+          <t>Emma Timmins‐Schiffman; Grace Crandall; Brent Vadopalas; Michael Riffle; Brook L. Nunn; Steven Roberts</t>
         </is>
       </c>
     </row>
@@ -1230,7 +1230,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Michael Riffle; Damon May; Molly P. Mikan; Daniel Jaschob; William Stafford Noble; Brook L. Nunn</t>
+          <t>Michael Riffle; Damon May; Emma Timmins‐Schiffman; Molly P. Mikan; Daniel Jaschob; William Stafford Noble; Brook L. Nunn</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1255,7 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Damon May; Molly P. Mikan; H. Rodger Harvey; Elhanan Borenstein; Brook L. Nunn; William Stafford Noble</t>
+          <t>Damon May; Emma Timmins‐Schiffman; Molly P. Mikan; H. Rodger Harvey; Elhanan Borenstein; Brook L. Nunn; William Stafford Noble</t>
         </is>
       </c>
     </row>
@@ -1280,7 +1280,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Damon May; Molly P. Mikan; Michael Riffle; Chris Frazar; H. Rodger Harvey; William Stafford Noble; Brook L. Nunn</t>
+          <t>Emma Timmins‐Schiffman; Damon May; Molly P. Mikan; Michael Riffle; Chris Frazar; H. Rodger Harvey; William Stafford Noble; Brook L. Nunn</t>
         </is>
       </c>
     </row>
@@ -1305,7 +1305,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Philip W. Boyd; Peter W. Dillingham; Christina M. McGraw; Edward A. Armstrong; Christopher E. Cornwall; Yuanyuan Feng; Catriona L. Hurd; Melanie Gault‐Ringold; Michael Y. Roleda; Brook L. Nunn</t>
+          <t>Philip W. Boyd; Peter W. Dillingham; Christina M. McGraw; Edward A. Armstrong; Christopher E. Cornwall; Yuanyuan Feng; Catriona L. Hurd; Melanie Gault‐Ringold; Michael Y. Roleda; Emma Timmins‐Schiffman; Brook L. Nunn</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1330,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Gary A. Winans; Nick Gayeski</t>
+          <t>Gary A. Winans; Nick Gayeski; Emma Timmins‐Schiffman</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1355,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Brook L. Nunn; Krystal Slattery; Karen A. Cameron; Karen Junge</t>
+          <t>Brook L. Nunn; Krystal Slattery; Karen A. Cameron; Emma Timmins‐Schiffman; Karen Junge</t>
         </is>
       </c>
     </row>
@@ -1380,7 +1380,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>William D Coffey; Wilber Hua; Brook L. Nunn; Gary H. Dickinson; Steven Roberts</t>
+          <t>Emma Timmins‐Schiffman; William D Coffey; Wilber Hua; Brook L. Nunn; Gary H. Dickinson; Steven Roberts</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1405,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Brook L. Nunn; David R. Goodlett; Steven Roberts</t>
+          <t>Emma Timmins‐Schiffman; Brook L. Nunn; David R. Goodlett; Steven Roberts</t>
         </is>
       </c>
     </row>
@@ -1430,7 +1430,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Steven Roberts</t>
+          <t>Emma Timmins‐Schiffman; Steven Roberts</t>
         </is>
       </c>
     </row>
@@ -1455,7 +1455,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Michael J. O’Donnell; Carolyn S. Friedman; Steven Roberts</t>
+          <t>Emma Timmins‐Schiffman; Michael J. O’Donnell; Carolyn S. Friedman; Steven Roberts</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Carolyn S. Friedman; Dave C. Metzger; Samuel J. White; Steven Roberts</t>
+          <t>Emma Timmins‐Schiffman; Carolyn S. Friedman; Dave C. Metzger; Samuel J. White; Steven Roberts</t>
         </is>
       </c>
     </row>

</xml_diff>